<commit_message>
Adicionada REC de ALP
</commit_message>
<xml_diff>
--- a/CST_ATP_2025.xlsx
+++ b/CST_ATP_2025.xlsx
@@ -390,10 +390,10 @@
       <c r="J1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>202510705410</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="2"/>
@@ -402,10 +402,10 @@
       <c r="I2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>202510705418</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="2"/>
@@ -418,10 +418,10 @@
       <c r="J3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>202510706076</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="2"/>
@@ -430,10 +430,10 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>202510706080</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="2" t="n">
@@ -450,10 +450,10 @@
       <c r="J5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>202510704356</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="2"/>
@@ -466,10 +466,10 @@
       <c r="J6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>202510704359</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="2" t="n">
@@ -486,10 +486,10 @@
       <c r="J7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>202510704126</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="n">
@@ -505,10 +505,10 @@
       <c r="I8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>202510706847</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="2"/>
@@ -521,10 +521,10 @@
       <c r="J9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>202510704129</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="2" t="n">
@@ -543,10 +543,10 @@
       <c r="J10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>202510704365</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="2" t="n">
@@ -563,10 +563,10 @@
       <c r="J11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>202510706125</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="2" t="n">
@@ -578,17 +578,19 @@
       <c r="E12" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F12" s="2"/>
+      <c r="F12" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>202510706135</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="2"/>
@@ -597,10 +599,10 @@
       <c r="I13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
+      <c r="A14" s="1" t="n">
         <v>202510706851</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="2" t="n">
@@ -619,27 +621,30 @@
       <c r="J14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="n">
+      <c r="A15" s="1" t="n">
         <v>202510704132</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="0" t="n">
+      <c r="C15" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E15" s="0" t="n">
+      <c r="E15" s="1" t="n">
         <v>2</v>
       </c>
+      <c r="F15" s="1" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="n">
+      <c r="A16" s="1" t="n">
         <v>202510704367</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C16" s="2" t="n">
@@ -652,10 +657,10 @@
       <c r="I16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="n">
+      <c r="A17" s="1" t="n">
         <v>202510704139</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="2" t="n">
@@ -667,244 +672,267 @@
       <c r="E17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="2"/>
+      <c r="F17" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="n">
+      <c r="A18" s="1" t="n">
         <v>202510706148</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="n">
+      <c r="A19" s="1" t="n">
         <v>202510704146</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="0" t="n">
+      <c r="C19" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D19" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="E19" s="0" t="n">
+      <c r="E19" s="1" t="n">
         <v>2</v>
       </c>
+      <c r="F19" s="1" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="n">
+      <c r="A20" s="1" t="n">
         <v>202510704369</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="0" t="n">
+      <c r="C20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D20" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="E20" s="0" t="n">
+      <c r="E20" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F20" s="1" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="n">
+      <c r="A21" s="1" t="n">
         <v>202510705420</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="0" t="n">
+      <c r="C21" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D21" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E21" s="0" t="n">
+      <c r="E21" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="n">
+      <c r="A22" s="1" t="n">
         <v>202510705417</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="E22" s="0" t="n">
+      <c r="C22" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E22" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="n">
+      <c r="A23" s="1" t="n">
         <v>202510706157</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="0" t="n">
+      <c r="C23" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D23" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="E23" s="0" t="n">
+      <c r="E23" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="F23" s="1" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="n">
+      <c r="A24" s="1" t="n">
         <v>202510704351</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="0" t="n">
+      <c r="C24" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D24" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="E24" s="0" t="n">
-        <v>6</v>
+      <c r="E24" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="n">
+      <c r="A25" s="1" t="n">
         <v>202510704374</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="E25" s="0" t="n">
+      <c r="C25" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F25" s="1" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="n">
+      <c r="A26" s="1" t="n">
         <v>202510704352</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="E26" s="0" t="n">
+      <c r="C26" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E26" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="n">
+      <c r="A27" s="1" t="n">
         <v>202510706162</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="0" t="n">
+      <c r="C27" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D27" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E27" s="0" t="n">
+      <c r="E27" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="n">
+      <c r="A28" s="1" t="n">
         <v>202510706165</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="0" t="n">
+      <c r="C28" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D28" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E28" s="0" t="n">
-        <v>4</v>
+      <c r="E28" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="n">
+      <c r="A29" s="1" t="n">
         <v>202510708629</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="n">
+      <c r="A30" s="1" t="n">
         <v>202510704353</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="0" t="n">
+      <c r="C30" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D30" s="1" t="n">
         <v>8</v>
       </c>
+      <c r="F30" s="1" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="n">
+      <c r="A31" s="1" t="n">
         <v>202310203444</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="n">
+      <c r="A32" s="1" t="n">
         <v>202510704376</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="B32" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="E32" s="0" t="n">
+      <c r="C32" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E32" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="n">
+      <c r="A33" s="1" t="n">
         <v>202510704380</v>
       </c>
-      <c r="B33" s="0" t="s">
+      <c r="B33" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="E33" s="0" t="n">
+      <c r="C33" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="n">
+      <c r="A34" s="1" t="n">
         <v>202510704354</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="B34" s="1" t="s">
         <v>38</v>
       </c>
       <c r="D34" s="1" t="n">
@@ -912,34 +940,40 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="n">
+      <c r="A35" s="1" t="n">
         <v>202510706174</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="B35" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="E35" s="0" t="n">
+      <c r="C35" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E35" s="1" t="n">
         <v>2</v>
       </c>
+      <c r="F35" s="1" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="n">
+      <c r="A36" s="1" t="n">
         <v>202510704355</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="B36" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="0" t="n">
+      <c r="C36" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D36" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E36" s="0" t="n">
+      <c r="E36" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="F36" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adicionado avaliação 3 de ATP
</commit_message>
<xml_diff>
--- a/CST_ATP_2025.xlsx
+++ b/CST_ATP_2025.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">Matricula</t>
   </si>
@@ -38,6 +38,12 @@
   </si>
   <si>
     <t xml:space="preserve">Recuperação 02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avaliação 03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recuperação 03</t>
   </si>
   <si>
     <t xml:space="preserve">ALEXANDRE BETEMPS MOHNSAM</t>
@@ -384,8 +390,12 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
     </row>
@@ -394,7 +404,7 @@
         <v>202510705410</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2"/>
       <c r="E2" s="2"/>
@@ -406,7 +416,7 @@
         <v>202510705418</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -422,7 +432,7 @@
         <v>202510706076</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" s="2"/>
       <c r="E4" s="2"/>
@@ -434,7 +444,7 @@
         <v>202510706080</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>8</v>
@@ -444,7 +454,9 @@
         <v>6</v>
       </c>
       <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+      <c r="G5" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -454,7 +466,7 @@
         <v>202510704356</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -470,7 +482,7 @@
         <v>202510704359</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>10</v>
@@ -480,7 +492,9 @@
         <v>6</v>
       </c>
       <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="G7" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -490,7 +504,7 @@
         <v>202510704126</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>6</v>
@@ -501,7 +515,9 @@
       <c r="E8" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="G8" s="2"/>
+      <c r="G8" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="I8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -509,7 +525,7 @@
         <v>202510706847</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -525,7 +541,7 @@
         <v>202510704129</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>6</v>
@@ -537,7 +553,9 @@
         <v>6</v>
       </c>
       <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="G10" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -547,7 +565,7 @@
         <v>202510704365</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>10</v>
@@ -557,7 +575,9 @@
         <v>10</v>
       </c>
       <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+      <c r="G11" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -567,7 +587,7 @@
         <v>202510706125</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>8</v>
@@ -581,7 +601,9 @@
       <c r="F12" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="2"/>
+      <c r="G12" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -591,7 +613,7 @@
         <v>202510706135</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C13" s="2"/>
       <c r="E13" s="2"/>
@@ -603,7 +625,7 @@
         <v>202510706851</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>8</v>
@@ -615,7 +637,9 @@
         <v>8</v>
       </c>
       <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="G14" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -625,7 +649,7 @@
         <v>202510704132</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>2</v>
@@ -638,6 +662,9 @@
       </c>
       <c r="F15" s="1" t="n">
         <v>4</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -645,7 +672,7 @@
         <v>202510704367</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>10</v>
@@ -653,7 +680,9 @@
       <c r="E16" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="G16" s="2"/>
+      <c r="G16" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="I16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -661,7 +690,7 @@
         <v>202510704139</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>6</v>
@@ -675,7 +704,9 @@
       <c r="F17" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="G17" s="2"/>
+      <c r="G17" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -685,7 +716,7 @@
         <v>202510706148</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -693,7 +724,7 @@
         <v>202510704146</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>4</v>
@@ -713,7 +744,7 @@
         <v>202510704369</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>4</v>
@@ -726,6 +757,9 @@
       </c>
       <c r="F20" s="1" t="n">
         <v>8</v>
+      </c>
+      <c r="G20" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -733,7 +767,7 @@
         <v>202510705420</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C21" s="1" t="n">
         <v>2</v>
@@ -742,6 +776,9 @@
         <v>2</v>
       </c>
       <c r="E21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -750,7 +787,7 @@
         <v>202510705417</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>10</v>
@@ -764,7 +801,7 @@
         <v>202510706157</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C23" s="1" t="n">
         <v>6</v>
@@ -777,6 +814,9 @@
       </c>
       <c r="F23" s="1" t="n">
         <v>8</v>
+      </c>
+      <c r="G23" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -784,7 +824,7 @@
         <v>202510704351</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C24" s="1" t="n">
         <v>6</v>
@@ -796,6 +836,9 @@
         <v>6</v>
       </c>
       <c r="F24" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="1" t="n">
         <v>2</v>
       </c>
     </row>
@@ -804,7 +847,7 @@
         <v>202510704374</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C25" s="1" t="n">
         <v>6</v>
@@ -814,6 +857,9 @@
       </c>
       <c r="F25" s="1" t="n">
         <v>8</v>
+      </c>
+      <c r="G25" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -821,13 +867,16 @@
         <v>202510704352</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C26" s="1" t="n">
         <v>10</v>
       </c>
       <c r="E26" s="1" t="n">
         <v>10</v>
+      </c>
+      <c r="G26" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -835,7 +884,7 @@
         <v>202510706162</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C27" s="1" t="n">
         <v>4</v>
@@ -845,6 +894,9 @@
       </c>
       <c r="E27" s="1" t="n">
         <v>10</v>
+      </c>
+      <c r="G27" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -852,7 +904,7 @@
         <v>202510706165</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C28" s="1" t="n">
         <v>4</v>
@@ -865,6 +917,9 @@
       </c>
       <c r="F28" s="1" t="n">
         <v>6</v>
+      </c>
+      <c r="G28" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -872,7 +927,7 @@
         <v>202510708629</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -880,7 +935,7 @@
         <v>202510704353</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C30" s="1" t="n">
         <v>6</v>
@@ -897,7 +952,10 @@
         <v>202310203444</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G31" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -905,12 +963,15 @@
         <v>202510704376</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C32" s="1" t="n">
         <v>10</v>
       </c>
       <c r="E32" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G32" s="1" t="n">
         <v>10</v>
       </c>
     </row>
@@ -919,13 +980,16 @@
         <v>202510704380</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C33" s="1" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="1" t="n">
         <v>10</v>
+      </c>
+      <c r="G33" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -933,10 +997,13 @@
         <v>202510704354</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D34" s="1" t="n">
         <v>10</v>
+      </c>
+      <c r="G34" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -944,7 +1011,7 @@
         <v>202510706174</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C35" s="1" t="n">
         <v>6</v>
@@ -954,6 +1021,9 @@
       </c>
       <c r="F35" s="1" t="n">
         <v>6</v>
+      </c>
+      <c r="G35" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -961,7 +1031,7 @@
         <v>202510704355</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C36" s="1" t="n">
         <v>4</v>
@@ -974,6 +1044,9 @@
       </c>
       <c r="F36" s="1" t="n">
         <v>6</v>
+      </c>
+      <c r="G36" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização planilhas e ajustes EDA
</commit_message>
<xml_diff>
--- a/CST_ATP_2025.xlsx
+++ b/CST_ATP_2025.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t xml:space="preserve">Matricula</t>
   </si>
@@ -44,6 +44,12 @@
   </si>
   <si>
     <t xml:space="preserve">Recuperação 03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avaliação 04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recuperação 04</t>
   </si>
   <si>
     <t xml:space="preserve">ALEXANDRE BETEMPS MOHNSAM</t>
@@ -396,15 +402,19 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>202510705410</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" s="2"/>
       <c r="E2" s="2"/>
@@ -416,7 +426,7 @@
         <v>202510705418</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -432,7 +442,7 @@
         <v>202510706076</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2"/>
       <c r="E4" s="2"/>
@@ -444,7 +454,7 @@
         <v>202510706080</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>8</v>
@@ -457,8 +467,12 @@
       <c r="G5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="H5" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="J5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -466,7 +480,7 @@
         <v>202510704356</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -482,7 +496,7 @@
         <v>202510704359</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>10</v>
@@ -496,7 +510,9 @@
         <v>10</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="I7" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="J7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -504,7 +520,7 @@
         <v>202510704126</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>6</v>
@@ -518,14 +534,16 @@
       <c r="G8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="I8" s="2"/>
+      <c r="I8" s="2" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>202510706847</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -541,7 +559,7 @@
         <v>202510704129</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>6</v>
@@ -556,8 +574,12 @@
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="H10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="J10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -565,7 +587,7 @@
         <v>202510704365</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>10</v>
@@ -579,7 +601,9 @@
         <v>10</v>
       </c>
       <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="I11" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="J11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -587,7 +611,7 @@
         <v>202510706125</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>8</v>
@@ -604,7 +628,9 @@
       <c r="G12" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="2"/>
+      <c r="H12" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
     </row>
@@ -613,7 +639,7 @@
         <v>202510706135</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C13" s="2"/>
       <c r="E13" s="2"/>
@@ -625,7 +651,7 @@
         <v>202510706851</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>8</v>
@@ -640,8 +666,12 @@
       <c r="G14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="H14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="J14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -649,7 +679,7 @@
         <v>202510704132</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>2</v>
@@ -665,6 +695,12 @@
       </c>
       <c r="G15" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H15" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I15" s="0" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -672,7 +708,7 @@
         <v>202510704367</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>10</v>
@@ -683,14 +719,16 @@
       <c r="G16" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="I16" s="2"/>
+      <c r="I16" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
         <v>202510704139</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>6</v>
@@ -707,8 +745,12 @@
       <c r="G17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
+      <c r="H17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="J17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -716,7 +758,7 @@
         <v>202510706148</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -724,7 +766,7 @@
         <v>202510704146</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>4</v>
@@ -737,6 +779,15 @@
       </c>
       <c r="F19" s="1" t="n">
         <v>4</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="I19" s="0" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -744,7 +795,7 @@
         <v>202510704369</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>4</v>
@@ -760,6 +811,9 @@
       </c>
       <c r="G20" s="1" t="n">
         <v>6</v>
+      </c>
+      <c r="I20" s="0" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -767,7 +821,7 @@
         <v>202510705420</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C21" s="1" t="n">
         <v>2</v>
@@ -780,6 +834,12 @@
       </c>
       <c r="G21" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="0" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -787,13 +847,22 @@
         <v>202510705417</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>10</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>10</v>
+      </c>
+      <c r="G22" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="H22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="0" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -801,7 +870,7 @@
         <v>202510706157</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C23" s="1" t="n">
         <v>6</v>
@@ -817,6 +886,12 @@
       </c>
       <c r="G23" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H23" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I23" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -824,7 +899,7 @@
         <v>202510704351</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C24" s="1" t="n">
         <v>6</v>
@@ -840,6 +915,12 @@
       </c>
       <c r="G24" s="1" t="n">
         <v>2</v>
+      </c>
+      <c r="H24" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I24" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -847,7 +928,7 @@
         <v>202510704374</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C25" s="1" t="n">
         <v>6</v>
@@ -860,6 +941,12 @@
       </c>
       <c r="G25" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H25" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="I25" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -867,7 +954,7 @@
         <v>202510704352</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C26" s="1" t="n">
         <v>10</v>
@@ -884,7 +971,7 @@
         <v>202510706162</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C27" s="1" t="n">
         <v>4</v>
@@ -897,6 +984,12 @@
       </c>
       <c r="G27" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H27" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="I27" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -904,7 +997,7 @@
         <v>202510706165</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C28" s="1" t="n">
         <v>4</v>
@@ -920,6 +1013,12 @@
       </c>
       <c r="G28" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H28" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I28" s="0" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -927,7 +1026,7 @@
         <v>202510708629</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -935,7 +1034,7 @@
         <v>202510704353</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C30" s="1" t="n">
         <v>6</v>
@@ -945,6 +1044,12 @@
       </c>
       <c r="F30" s="1" t="n">
         <v>8</v>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="I30" s="0" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -952,7 +1057,7 @@
         <v>202310203444</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G31" s="1" t="n">
         <v>0</v>
@@ -963,7 +1068,7 @@
         <v>202510704376</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C32" s="1" t="n">
         <v>10</v>
@@ -972,6 +1077,9 @@
         <v>10</v>
       </c>
       <c r="G32" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I32" s="0" t="n">
         <v>10</v>
       </c>
     </row>
@@ -980,7 +1088,7 @@
         <v>202510704380</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C33" s="1" t="n">
         <v>6</v>
@@ -990,6 +1098,9 @@
       </c>
       <c r="G33" s="1" t="n">
         <v>2</v>
+      </c>
+      <c r="I33" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -997,13 +1108,19 @@
         <v>202510704354</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D34" s="1" t="n">
         <v>10</v>
       </c>
       <c r="G34" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H34" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I34" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1011,7 +1128,7 @@
         <v>202510706174</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C35" s="1" t="n">
         <v>6</v>
@@ -1024,6 +1141,12 @@
       </c>
       <c r="G35" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H35" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I35" s="0" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1031,7 +1154,7 @@
         <v>202510704355</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C36" s="1" t="n">
         <v>4</v>
@@ -1047,6 +1170,12 @@
       </c>
       <c r="G36" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I36" s="0" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>